<commit_message>
feat: lp register updated, pyrfc not working
</commit_message>
<xml_diff>
--- a/08 - Excels/Cadastro-LPs.xlsx
+++ b/08 - Excels/Cadastro-LPs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFC4658-EA3F-4609-9E66-6E0F5AFBD251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA881D8C-06BD-48CF-B7A7-90B24657086D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,12 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Status</t>
   </si>
   <si>
     <t>PM</t>
+  </si>
+  <si>
+    <t>000014153774</t>
   </si>
 </sst>
 </file>
@@ -54,7 +57,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -77,11 +80,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -91,6 +109,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -394,24 +415,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>14149511</v>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: LP Register bot created
</commit_message>
<xml_diff>
--- a/08 - Excels/Cadastro-LPs.xlsx
+++ b/08 - Excels/Cadastro-LPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\08 - Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA881D8C-06BD-48CF-B7A7-90B24657086D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00C43BC3-4D4D-4217-BCC2-BD3D7B784A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,22 +20,70 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>PM</t>
-  </si>
-  <si>
-    <t>000014153774</t>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>4713400000</t>
+  </si>
+  <si>
+    <t>685531</t>
+  </si>
+  <si>
+    <t>LP-054431</t>
+  </si>
+  <si>
+    <t>Objeto de Liquidação</t>
+  </si>
+  <si>
+    <t>Part Number</t>
+  </si>
+  <si>
+    <t>Rodrigo Melo</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>Novo - Série 0196</t>
+  </si>
+  <si>
+    <t>QMM</t>
+  </si>
+  <si>
+    <t>Prazo Final</t>
+  </si>
+  <si>
+    <t>Quantidade</t>
+  </si>
+  <si>
+    <t>Denominação</t>
+  </si>
+  <si>
+    <t>Entregar para</t>
+  </si>
+  <si>
+    <t>Custo estimado</t>
+  </si>
+  <si>
+    <t>Elemento PEP</t>
+  </si>
+  <si>
+    <t>Esquema de Alocação</t>
+  </si>
+  <si>
+    <t>Responsável</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -48,6 +96,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -57,7 +111,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -80,38 +134,29 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -415,25 +460,93 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>46027</v>
+      </c>
+      <c r="B2" s="4">
+        <v>46125</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>2</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="5">
+        <v>2000</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>